<commit_message>
fix: corregir scorecard para usar endpoint anchor y superar limite de 1000 registros de Supabase
</commit_message>
<xml_diff>
--- a/Libro1.xlsx
+++ b/Libro1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julpa\OneDrive\Desktop\devaluacion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julpa\OneDrive\Desktop\Proyecto de cambio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B5A9A97-EF1D-4A74-A77C-A02BA7E7FDC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18E77DA7-7055-4C6D-9585-7FF8683C0B3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A65F3A25-362E-496A-B2FF-A0D876B66B4D}"/>
   </bookViews>
@@ -10376,22 +10376,22 @@
         <v>46233</v>
       </c>
       <c r="C374" s="16">
-        <v>737.88</v>
+        <v>745.63</v>
       </c>
       <c r="D374" s="16">
-        <v>841.84</v>
+        <v>848.82</v>
       </c>
       <c r="E374" s="16">
         <v>863.78</v>
       </c>
       <c r="F374" s="23"/>
       <c r="G374" s="17">
-        <f t="shared" ref="G374:G387" si="35">(E374-C374)/C374</f>
-        <v>0.17062394969371711</v>
+        <f t="shared" ref="G374:G386" si="35">(E374-C374)/C374</f>
+        <v>0.15845660716441126</v>
       </c>
       <c r="H374" s="17">
-        <f t="shared" ref="H374:H387" si="36">(E374-D374)/D374</f>
-        <v>2.6061959517247862E-2</v>
+        <f t="shared" ref="H374:H386" si="36">(E374-D374)/D374</f>
+        <v>1.7624466907000213E-2</v>
       </c>
     </row>
     <row r="375" spans="1:10" x14ac:dyDescent="0.3">
@@ -10402,10 +10402,10 @@
         <v>46234</v>
       </c>
       <c r="C375" s="16">
-        <v>737.88</v>
+        <v>746.62</v>
       </c>
       <c r="D375" s="16">
-        <v>841.84</v>
+        <v>858.98</v>
       </c>
       <c r="E375" s="16">
         <v>851.49</v>
@@ -10413,11 +10413,11 @@
       <c r="F375" s="24"/>
       <c r="G375" s="17">
         <f t="shared" si="35"/>
-        <v>0.15396812489835748</v>
+        <v>0.14045967158661701</v>
       </c>
       <c r="H375" s="17">
         <f t="shared" si="36"/>
-        <v>1.1462985840539742E-2</v>
+        <v>-8.7196442292020865E-3</v>
       </c>
     </row>
     <row r="376" spans="1:10" x14ac:dyDescent="0.3">
@@ -10428,10 +10428,10 @@
         <v>46234</v>
       </c>
       <c r="C376" s="16">
-        <v>742.22</v>
+        <v>746.62</v>
       </c>
       <c r="D376" s="16">
-        <v>844.21</v>
+        <v>858.98</v>
       </c>
       <c r="E376" s="12">
         <v>852.24</v>
@@ -10439,11 +10439,11 @@
       <c r="F376" s="23"/>
       <c r="G376" s="14">
         <f t="shared" si="35"/>
-        <v>0.14823098272749316</v>
+        <v>0.1414641986552731</v>
       </c>
       <c r="H376" s="14">
         <f t="shared" si="36"/>
-        <v>9.5118513166155012E-3</v>
+        <v>-7.8465156348227066E-3</v>
       </c>
       <c r="J376" s="15"/>
     </row>
@@ -10455,10 +10455,10 @@
         <v>46235</v>
       </c>
       <c r="C377" s="16">
-        <v>742.22</v>
+        <v>746.62</v>
       </c>
       <c r="D377" s="16">
-        <v>844.21</v>
+        <v>861.18</v>
       </c>
       <c r="E377" s="12">
         <v>850.91</v>
@@ -10466,11 +10466,11 @@
       <c r="F377" s="24"/>
       <c r="G377" s="14">
         <f t="shared" si="35"/>
-        <v>0.14643906119479391</v>
+        <v>0.1396828373201896</v>
       </c>
       <c r="H377" s="14">
         <f t="shared" si="36"/>
-        <v>7.9364139254450104E-3</v>
+        <v>-1.1925497573097358E-2</v>
       </c>
       <c r="J377" s="11"/>
     </row>
@@ -10478,14 +10478,14 @@
       <c r="A378" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B378" s="11">
-        <v>46236</v>
+      <c r="B378" s="15">
+        <v>46235</v>
       </c>
       <c r="C378" s="16">
-        <v>742.22</v>
+        <v>746.62</v>
       </c>
       <c r="D378" s="16">
-        <v>844.21</v>
+        <v>861.18</v>
       </c>
       <c r="E378" s="12">
         <v>856.11</v>
@@ -10493,11 +10493,11 @@
       <c r="F378" s="22"/>
       <c r="G378" s="14">
         <f t="shared" si="35"/>
-        <v>0.15344507019482093</v>
+        <v>0.14664755832953846</v>
       </c>
       <c r="H378" s="14">
         <f t="shared" si="36"/>
-        <v>1.409601876310394E-2</v>
+        <v>-5.8872709538074931E-3</v>
       </c>
       <c r="J378" s="15"/>
     </row>
@@ -10505,14 +10505,14 @@
       <c r="A379" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B379" s="15">
-        <v>46235</v>
+      <c r="B379" s="11">
+        <v>46236</v>
       </c>
       <c r="C379" s="16">
-        <v>742.22</v>
+        <v>746.62</v>
       </c>
       <c r="D379" s="16">
-        <v>844.21</v>
+        <v>861.18</v>
       </c>
       <c r="E379" s="12">
         <v>846.34</v>
@@ -10520,11 +10520,11 @@
       <c r="F379" s="22"/>
       <c r="G379" s="14">
         <f t="shared" si="35"/>
-        <v>0.14028185713130878</v>
+        <v>0.133561919048512</v>
       </c>
       <c r="H379" s="14">
         <f t="shared" si="36"/>
-        <v>2.5230689046564191E-3</v>
+        <v>-1.72321698135116E-2</v>
       </c>
       <c r="J379" s="15"/>
     </row>
@@ -10532,14 +10532,14 @@
       <c r="A380" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B380" s="15">
-        <v>46235</v>
+      <c r="B380" s="11">
+        <v>46236</v>
       </c>
       <c r="C380" s="16">
-        <v>742.22</v>
+        <v>746.62</v>
       </c>
       <c r="D380" s="16">
-        <v>844.21</v>
+        <v>861.18</v>
       </c>
       <c r="E380" s="12">
         <v>847.52</v>
@@ -10547,11 +10547,11 @@
       <c r="F380" s="22"/>
       <c r="G380" s="14">
         <f t="shared" si="35"/>
-        <v>0.14187168225054558</v>
+        <v>0.13514237496986414</v>
       </c>
       <c r="H380" s="14">
         <f t="shared" si="36"/>
-        <v>3.9208253870481819E-3</v>
+        <v>-1.5861956849903585E-2</v>
       </c>
       <c r="J380" s="11"/>
     </row>
@@ -10559,14 +10559,14 @@
       <c r="A381" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B381" s="11">
-        <v>46236</v>
+      <c r="B381" s="15">
+        <v>46237</v>
       </c>
       <c r="C381" s="16">
-        <v>742.22</v>
+        <v>744.78</v>
       </c>
       <c r="D381" s="16">
-        <v>844.21</v>
+        <v>861.18</v>
       </c>
       <c r="E381" s="12">
         <v>847.43</v>
@@ -10574,11 +10574,11 @@
       <c r="F381" s="22"/>
       <c r="G381" s="14">
         <f t="shared" si="35"/>
-        <v>0.14175042440246816</v>
+        <v>0.13782593517548805</v>
       </c>
       <c r="H381" s="14">
         <f t="shared" si="36"/>
-        <v>3.8142168417809709E-3</v>
+        <v>-1.5966464618314406E-2</v>
       </c>
       <c r="J381" s="11"/>
     </row>
@@ -10586,14 +10586,14 @@
       <c r="A382" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B382" s="11">
-        <v>46236</v>
+      <c r="B382" s="15">
+        <v>46237</v>
       </c>
       <c r="C382" s="16">
-        <v>742.22</v>
+        <v>744.78</v>
       </c>
       <c r="D382" s="16">
-        <v>844.21</v>
+        <v>861.18</v>
       </c>
       <c r="E382" s="12">
         <v>852.49</v>
@@ -10601,11 +10601,11 @@
       <c r="F382" s="22"/>
       <c r="G382" s="14">
         <f t="shared" si="35"/>
-        <v>0.1485678100832637</v>
+        <v>0.14461988775208792</v>
       </c>
       <c r="H382" s="14">
         <f t="shared" si="36"/>
-        <v>9.80798616457987E-3</v>
+        <v>-1.0090805638774637E-2</v>
       </c>
       <c r="J382" s="15"/>
     </row>
@@ -10613,14 +10613,14 @@
       <c r="A383" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B383" s="15">
-        <v>46237</v>
+      <c r="B383" s="11">
+        <v>46238</v>
       </c>
       <c r="C383" s="16">
-        <v>742.81</v>
+        <v>752.09</v>
       </c>
       <c r="D383" s="16">
-        <v>844.75</v>
+        <v>865.17</v>
       </c>
       <c r="E383" s="12">
         <v>840.78</v>
@@ -10628,11 +10628,11 @@
       <c r="F383" s="22"/>
       <c r="G383" s="14">
         <f t="shared" si="35"/>
-        <v>0.13189106231741635</v>
+        <v>0.11792471645680695</v>
       </c>
       <c r="H383" s="14">
         <f t="shared" si="36"/>
-        <v>-4.699615270790207E-3</v>
+        <v>-2.8190991365858717E-2</v>
       </c>
       <c r="J383" s="15"/>
     </row>
@@ -10640,14 +10640,14 @@
       <c r="A384" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B384" s="15">
-        <v>46237</v>
-      </c>
-      <c r="C384" s="12">
-        <v>742.81</v>
-      </c>
-      <c r="D384" s="12">
-        <v>844.75</v>
+      <c r="B384" s="11">
+        <v>46238</v>
+      </c>
+      <c r="C384" s="16">
+        <v>752.09</v>
+      </c>
+      <c r="D384" s="16">
+        <v>865.17</v>
       </c>
       <c r="E384" s="12">
         <v>843.83</v>
@@ -10655,11 +10655,11 @@
       <c r="F384" s="22"/>
       <c r="G384" s="14">
         <f t="shared" si="35"/>
-        <v>0.13599709212315411</v>
+        <v>0.12198008217101677</v>
       </c>
       <c r="H384" s="14">
         <f t="shared" si="36"/>
-        <v>-1.0890796093518309E-3</v>
+        <v>-2.4665672642370771E-2</v>
       </c>
       <c r="J384" s="11"/>
     </row>
@@ -10668,13 +10668,13 @@
         <v>9</v>
       </c>
       <c r="B385" s="11">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C385" s="12">
-        <v>744.22</v>
+        <v>755.15</v>
       </c>
       <c r="D385" s="12">
-        <v>846.07</v>
+        <v>870.04</v>
       </c>
       <c r="E385" s="12">
         <v>846.16</v>
@@ -10682,11 +10682,11 @@
       <c r="F385" s="22"/>
       <c r="G385" s="14">
         <f t="shared" si="35"/>
-        <v>0.13697562548708705</v>
+        <v>0.12051910216513274</v>
       </c>
       <c r="H385" s="14">
         <f t="shared" si="36"/>
-        <v>1.0637417707745003E-4</v>
+        <v>-2.7447013930394001E-2</v>
       </c>
       <c r="J385" s="11"/>
     </row>
@@ -10695,13 +10695,13 @@
         <v>10</v>
       </c>
       <c r="B386" s="11">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C386" s="12">
-        <v>744.22</v>
+        <v>755.15</v>
       </c>
       <c r="D386" s="12">
-        <v>846.07</v>
+        <v>870.04</v>
       </c>
       <c r="E386" s="16">
         <v>843.8</v>
@@ -10709,11 +10709,11 @@
       <c r="F386" s="22"/>
       <c r="G386" s="17">
         <f t="shared" si="35"/>
-        <v>0.1338045201687672</v>
+        <v>0.1173938952525988</v>
       </c>
       <c r="H386" s="20">
         <f t="shared" si="36"/>
-        <v>-2.6829931329560145E-3</v>
+        <v>-3.015953289503932E-2</v>
       </c>
       <c r="J386" s="11"/>
     </row>
@@ -10729,6 +10729,138 @@
     </row>
   </sheetData>
   <mergeCells count="156">
+    <mergeCell ref="F363:F364"/>
+    <mergeCell ref="F365:F366"/>
+    <mergeCell ref="F367:F368"/>
+    <mergeCell ref="F369:F370"/>
+    <mergeCell ref="F371:F372"/>
+    <mergeCell ref="F350:F351"/>
+    <mergeCell ref="F352:F353"/>
+    <mergeCell ref="F354:F355"/>
+    <mergeCell ref="F357:F358"/>
+    <mergeCell ref="F359:F360"/>
+    <mergeCell ref="F361:F362"/>
+    <mergeCell ref="F338:F339"/>
+    <mergeCell ref="F340:F341"/>
+    <mergeCell ref="F342:F343"/>
+    <mergeCell ref="F344:F345"/>
+    <mergeCell ref="F346:F347"/>
+    <mergeCell ref="F348:F349"/>
+    <mergeCell ref="F326:F327"/>
+    <mergeCell ref="F328:F329"/>
+    <mergeCell ref="F330:F331"/>
+    <mergeCell ref="F332:F333"/>
+    <mergeCell ref="F334:F335"/>
+    <mergeCell ref="F336:F337"/>
+    <mergeCell ref="F314:F315"/>
+    <mergeCell ref="F316:F317"/>
+    <mergeCell ref="F318:F319"/>
+    <mergeCell ref="F320:F321"/>
+    <mergeCell ref="F322:F323"/>
+    <mergeCell ref="F324:F325"/>
+    <mergeCell ref="F302:F303"/>
+    <mergeCell ref="F304:F305"/>
+    <mergeCell ref="F306:F307"/>
+    <mergeCell ref="F308:F309"/>
+    <mergeCell ref="F310:F311"/>
+    <mergeCell ref="F312:F313"/>
+    <mergeCell ref="F290:F291"/>
+    <mergeCell ref="F292:F293"/>
+    <mergeCell ref="F294:F295"/>
+    <mergeCell ref="F296:F297"/>
+    <mergeCell ref="F298:F299"/>
+    <mergeCell ref="F300:F301"/>
+    <mergeCell ref="F277:F278"/>
+    <mergeCell ref="F279:F280"/>
+    <mergeCell ref="F281:F282"/>
+    <mergeCell ref="F283:F284"/>
+    <mergeCell ref="F285:F286"/>
+    <mergeCell ref="F287:F288"/>
+    <mergeCell ref="F265:F266"/>
+    <mergeCell ref="F267:F268"/>
+    <mergeCell ref="F269:F270"/>
+    <mergeCell ref="F271:F272"/>
+    <mergeCell ref="F273:F274"/>
+    <mergeCell ref="F275:F276"/>
+    <mergeCell ref="F253:F254"/>
+    <mergeCell ref="F255:F256"/>
+    <mergeCell ref="F257:F258"/>
+    <mergeCell ref="F259:F260"/>
+    <mergeCell ref="F261:F262"/>
+    <mergeCell ref="F263:F264"/>
+    <mergeCell ref="F240:F241"/>
+    <mergeCell ref="F242:F243"/>
+    <mergeCell ref="F244:F245"/>
+    <mergeCell ref="F246:F247"/>
+    <mergeCell ref="F248:F249"/>
+    <mergeCell ref="F250:F251"/>
+    <mergeCell ref="F227:F228"/>
+    <mergeCell ref="F229:F230"/>
+    <mergeCell ref="F231:F232"/>
+    <mergeCell ref="F233:F234"/>
+    <mergeCell ref="F235:F236"/>
+    <mergeCell ref="F238:F239"/>
+    <mergeCell ref="F214:F215"/>
+    <mergeCell ref="F216:F217"/>
+    <mergeCell ref="F218:F219"/>
+    <mergeCell ref="F220:F221"/>
+    <mergeCell ref="F223:F224"/>
+    <mergeCell ref="F225:F226"/>
+    <mergeCell ref="F202:F203"/>
+    <mergeCell ref="F204:F205"/>
+    <mergeCell ref="F206:F207"/>
+    <mergeCell ref="F208:F209"/>
+    <mergeCell ref="F210:F211"/>
+    <mergeCell ref="F212:F213"/>
+    <mergeCell ref="F190:F191"/>
+    <mergeCell ref="F192:F193"/>
+    <mergeCell ref="F194:F195"/>
+    <mergeCell ref="F196:F197"/>
+    <mergeCell ref="F198:F199"/>
+    <mergeCell ref="F200:F201"/>
+    <mergeCell ref="F177:F178"/>
+    <mergeCell ref="F180:F181"/>
+    <mergeCell ref="F182:F183"/>
+    <mergeCell ref="F184:F185"/>
+    <mergeCell ref="F186:F187"/>
+    <mergeCell ref="F188:F189"/>
+    <mergeCell ref="F165:F166"/>
+    <mergeCell ref="F167:F168"/>
+    <mergeCell ref="F169:F170"/>
+    <mergeCell ref="F171:F172"/>
+    <mergeCell ref="F173:F174"/>
+    <mergeCell ref="F175:F176"/>
+    <mergeCell ref="F152:F153"/>
+    <mergeCell ref="F154:F155"/>
+    <mergeCell ref="F156:F157"/>
+    <mergeCell ref="F158:F159"/>
+    <mergeCell ref="F160:F161"/>
+    <mergeCell ref="F162:F163"/>
+    <mergeCell ref="F139:F140"/>
+    <mergeCell ref="F141:F142"/>
+    <mergeCell ref="F143:F144"/>
+    <mergeCell ref="F145:F146"/>
+    <mergeCell ref="F147:F148"/>
+    <mergeCell ref="F150:F151"/>
+    <mergeCell ref="F126:F127"/>
+    <mergeCell ref="F128:F129"/>
+    <mergeCell ref="F130:F131"/>
+    <mergeCell ref="F132:F133"/>
+    <mergeCell ref="F135:F136"/>
+    <mergeCell ref="F137:F138"/>
+    <mergeCell ref="F85:F86"/>
+    <mergeCell ref="F113:F114"/>
+    <mergeCell ref="F115:F116"/>
+    <mergeCell ref="F117:F118"/>
+    <mergeCell ref="F120:F121"/>
+    <mergeCell ref="F122:F123"/>
+    <mergeCell ref="F124:F125"/>
+    <mergeCell ref="F100:F101"/>
+    <mergeCell ref="F102:F103"/>
+    <mergeCell ref="F105:F106"/>
+    <mergeCell ref="F107:F108"/>
+    <mergeCell ref="F109:F110"/>
+    <mergeCell ref="F111:F112"/>
     <mergeCell ref="F380:F381"/>
     <mergeCell ref="F382:F383"/>
     <mergeCell ref="F384:F385"/>
@@ -10753,138 +10885,6 @@
     <mergeCell ref="F79:F80"/>
     <mergeCell ref="F81:F82"/>
     <mergeCell ref="F83:F84"/>
-    <mergeCell ref="F85:F86"/>
-    <mergeCell ref="F113:F114"/>
-    <mergeCell ref="F115:F116"/>
-    <mergeCell ref="F117:F118"/>
-    <mergeCell ref="F120:F121"/>
-    <mergeCell ref="F122:F123"/>
-    <mergeCell ref="F124:F125"/>
-    <mergeCell ref="F100:F101"/>
-    <mergeCell ref="F102:F103"/>
-    <mergeCell ref="F105:F106"/>
-    <mergeCell ref="F107:F108"/>
-    <mergeCell ref="F109:F110"/>
-    <mergeCell ref="F111:F112"/>
-    <mergeCell ref="F139:F140"/>
-    <mergeCell ref="F141:F142"/>
-    <mergeCell ref="F143:F144"/>
-    <mergeCell ref="F145:F146"/>
-    <mergeCell ref="F147:F148"/>
-    <mergeCell ref="F150:F151"/>
-    <mergeCell ref="F126:F127"/>
-    <mergeCell ref="F128:F129"/>
-    <mergeCell ref="F130:F131"/>
-    <mergeCell ref="F132:F133"/>
-    <mergeCell ref="F135:F136"/>
-    <mergeCell ref="F137:F138"/>
-    <mergeCell ref="F165:F166"/>
-    <mergeCell ref="F167:F168"/>
-    <mergeCell ref="F169:F170"/>
-    <mergeCell ref="F171:F172"/>
-    <mergeCell ref="F173:F174"/>
-    <mergeCell ref="F175:F176"/>
-    <mergeCell ref="F152:F153"/>
-    <mergeCell ref="F154:F155"/>
-    <mergeCell ref="F156:F157"/>
-    <mergeCell ref="F158:F159"/>
-    <mergeCell ref="F160:F161"/>
-    <mergeCell ref="F162:F163"/>
-    <mergeCell ref="F190:F191"/>
-    <mergeCell ref="F192:F193"/>
-    <mergeCell ref="F194:F195"/>
-    <mergeCell ref="F196:F197"/>
-    <mergeCell ref="F198:F199"/>
-    <mergeCell ref="F200:F201"/>
-    <mergeCell ref="F177:F178"/>
-    <mergeCell ref="F180:F181"/>
-    <mergeCell ref="F182:F183"/>
-    <mergeCell ref="F184:F185"/>
-    <mergeCell ref="F186:F187"/>
-    <mergeCell ref="F188:F189"/>
-    <mergeCell ref="F214:F215"/>
-    <mergeCell ref="F216:F217"/>
-    <mergeCell ref="F218:F219"/>
-    <mergeCell ref="F220:F221"/>
-    <mergeCell ref="F223:F224"/>
-    <mergeCell ref="F225:F226"/>
-    <mergeCell ref="F202:F203"/>
-    <mergeCell ref="F204:F205"/>
-    <mergeCell ref="F206:F207"/>
-    <mergeCell ref="F208:F209"/>
-    <mergeCell ref="F210:F211"/>
-    <mergeCell ref="F212:F213"/>
-    <mergeCell ref="F240:F241"/>
-    <mergeCell ref="F242:F243"/>
-    <mergeCell ref="F244:F245"/>
-    <mergeCell ref="F246:F247"/>
-    <mergeCell ref="F248:F249"/>
-    <mergeCell ref="F250:F251"/>
-    <mergeCell ref="F227:F228"/>
-    <mergeCell ref="F229:F230"/>
-    <mergeCell ref="F231:F232"/>
-    <mergeCell ref="F233:F234"/>
-    <mergeCell ref="F235:F236"/>
-    <mergeCell ref="F238:F239"/>
-    <mergeCell ref="F265:F266"/>
-    <mergeCell ref="F267:F268"/>
-    <mergeCell ref="F269:F270"/>
-    <mergeCell ref="F271:F272"/>
-    <mergeCell ref="F273:F274"/>
-    <mergeCell ref="F275:F276"/>
-    <mergeCell ref="F253:F254"/>
-    <mergeCell ref="F255:F256"/>
-    <mergeCell ref="F257:F258"/>
-    <mergeCell ref="F259:F260"/>
-    <mergeCell ref="F261:F262"/>
-    <mergeCell ref="F263:F264"/>
-    <mergeCell ref="F290:F291"/>
-    <mergeCell ref="F292:F293"/>
-    <mergeCell ref="F294:F295"/>
-    <mergeCell ref="F296:F297"/>
-    <mergeCell ref="F298:F299"/>
-    <mergeCell ref="F300:F301"/>
-    <mergeCell ref="F277:F278"/>
-    <mergeCell ref="F279:F280"/>
-    <mergeCell ref="F281:F282"/>
-    <mergeCell ref="F283:F284"/>
-    <mergeCell ref="F285:F286"/>
-    <mergeCell ref="F287:F288"/>
-    <mergeCell ref="F314:F315"/>
-    <mergeCell ref="F316:F317"/>
-    <mergeCell ref="F318:F319"/>
-    <mergeCell ref="F320:F321"/>
-    <mergeCell ref="F322:F323"/>
-    <mergeCell ref="F324:F325"/>
-    <mergeCell ref="F302:F303"/>
-    <mergeCell ref="F304:F305"/>
-    <mergeCell ref="F306:F307"/>
-    <mergeCell ref="F308:F309"/>
-    <mergeCell ref="F310:F311"/>
-    <mergeCell ref="F312:F313"/>
-    <mergeCell ref="F338:F339"/>
-    <mergeCell ref="F340:F341"/>
-    <mergeCell ref="F342:F343"/>
-    <mergeCell ref="F344:F345"/>
-    <mergeCell ref="F346:F347"/>
-    <mergeCell ref="F348:F349"/>
-    <mergeCell ref="F326:F327"/>
-    <mergeCell ref="F328:F329"/>
-    <mergeCell ref="F330:F331"/>
-    <mergeCell ref="F332:F333"/>
-    <mergeCell ref="F334:F335"/>
-    <mergeCell ref="F336:F337"/>
-    <mergeCell ref="F363:F364"/>
-    <mergeCell ref="F365:F366"/>
-    <mergeCell ref="F367:F368"/>
-    <mergeCell ref="F369:F370"/>
-    <mergeCell ref="F371:F372"/>
-    <mergeCell ref="F350:F351"/>
-    <mergeCell ref="F352:F353"/>
-    <mergeCell ref="F354:F355"/>
-    <mergeCell ref="F357:F358"/>
-    <mergeCell ref="F359:F360"/>
-    <mergeCell ref="F361:F362"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>